<commit_message>
app.py was created, it allows streamlit local running, in adition, AccionesColombia,ipynb incorporates a stock plot/summarize display in the same cell for all stocks.
</commit_message>
<xml_diff>
--- a/Data/colombia_company_data/table_Input.xlsx
+++ b/Data/colombia_company_data/table_Input.xlsx
@@ -10,7 +10,7 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="192" documentId="8_{508D59E9-383F-477D-B14D-D49FBC91448D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B1114F42-AA72-445B-96CB-A04456BB496D}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{D401B9FE-6600-4CE7-9513-628A64DF9DCD}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{D401B9FE-6600-4CE7-9513-628A64DF9DCD}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -543,17 +543,17 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{44E29657-2344-47A0-829E-199EFDF79B4F}">
   <dimension ref="A1:R9"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="22.453125" customWidth="1"/>
-    <col min="2" max="2" width="19.7265625" customWidth="1"/>
-    <col min="3" max="3" width="14.453125" customWidth="1"/>
+    <col min="1" max="1" width="22.42578125" customWidth="1"/>
+    <col min="2" max="2" width="19.7109375" customWidth="1"/>
+    <col min="3" max="3" width="14.42578125" customWidth="1"/>
     <col min="7" max="7" width="12" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="12" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="15.26953125" customWidth="1"/>
+    <col min="12" max="12" width="15.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:18" x14ac:dyDescent="0.25">
       <c r="B1" t="s">
         <v>6</v>
       </c>
@@ -606,7 +606,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="2" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>38</v>
       </c>
@@ -662,7 +662,7 @@
         <v>46247</v>
       </c>
     </row>
-    <row r="3" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>1</v>
       </c>
@@ -718,7 +718,7 @@
         <v>116601012</v>
       </c>
     </row>
-    <row r="4" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>2</v>
       </c>
@@ -774,7 +774,7 @@
         <v>31474.22</v>
       </c>
     </row>
-    <row r="5" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>3</v>
       </c>
@@ -830,7 +830,7 @@
         <v>0.78</v>
       </c>
     </row>
-    <row r="6" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>4</v>
       </c>
@@ -886,7 +886,7 @@
         <v>5.68</v>
       </c>
     </row>
-    <row r="7" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>5</v>
       </c>
@@ -942,7 +942,7 @@
         <v>4338.8</v>
       </c>
     </row>
-    <row r="8" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>29</v>
       </c>
@@ -998,7 +998,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>24</v>
       </c>

</xml_diff>

<commit_message>
Davivienda fair stock price and suggestions was added to company table, stock data was updated
</commit_message>
<xml_diff>
--- a/Data/colombia_company_data/table_Input.xlsx
+++ b/Data/colombia_company_data/table_Input.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://parexresources-my.sharepoint.com/personal/ypalacios_parexresources_com/Documents/Documents/Github Projects/Colombia_finance/Data/colombia_company_data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="192" documentId="8_{508D59E9-383F-477D-B14D-D49FBC91448D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B1114F42-AA72-445B-96CB-A04456BB496D}"/>
+  <xr:revisionPtr revIDLastSave="234" documentId="8_{508D59E9-383F-477D-B14D-D49FBC91448D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1719D265-F77C-49EC-B233-697229837D80}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{D401B9FE-6600-4CE7-9513-628A64DF9DCD}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="45">
   <si>
     <t>CELSIA</t>
   </si>
@@ -159,6 +159,21 @@
   </si>
   <si>
     <t>https://www.bvc.com.co/renta-variable-mercado-local/pfdavvnda?tab=resumen</t>
+  </si>
+  <si>
+    <t>Davivienda's Fair Price</t>
+  </si>
+  <si>
+    <t>Davivienda's Suggest</t>
+  </si>
+  <si>
+    <t>BUY</t>
+  </si>
+  <si>
+    <t>KEEP</t>
+  </si>
+  <si>
+    <t>SELL</t>
   </si>
 </sst>
 </file>
@@ -542,7 +557,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{44E29657-2344-47A0-829E-199EFDF79B4F}">
-  <dimension ref="A1:R9"/>
+  <dimension ref="A1:R11"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="22.42578125" customWidth="1"/>
@@ -776,303 +791,385 @@
     </row>
     <row r="5" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>3</v>
-      </c>
-      <c r="B5">
-        <v>0.89</v>
+        <v>40</v>
       </c>
       <c r="C5">
-        <v>1.2</v>
+        <v>6100</v>
       </c>
       <c r="D5">
-        <v>1.34</v>
+        <v>12500</v>
       </c>
       <c r="E5">
-        <v>1.94</v>
+        <v>74800</v>
       </c>
       <c r="F5">
-        <v>0.59</v>
+        <v>26900</v>
       </c>
       <c r="G5">
-        <v>1.37</v>
+        <v>2400</v>
       </c>
       <c r="H5">
-        <v>1.5</v>
+        <v>3900</v>
       </c>
       <c r="I5">
-        <v>1.28</v>
+        <v>18100</v>
       </c>
       <c r="J5">
-        <v>1.06</v>
+        <v>890</v>
       </c>
       <c r="K5">
-        <v>1.21</v>
+        <v>71300</v>
       </c>
       <c r="L5">
-        <v>0.98</v>
+        <v>62800</v>
       </c>
       <c r="M5">
-        <v>1.91</v>
-      </c>
-      <c r="N5">
-        <v>17.649999999999999</v>
-      </c>
-      <c r="O5">
-        <v>1.1100000000000001</v>
-      </c>
-      <c r="P5">
-        <v>1.43</v>
+        <v>27500</v>
       </c>
       <c r="Q5">
-        <v>1.94</v>
-      </c>
-      <c r="R5">
-        <v>0.78</v>
+        <v>69200</v>
       </c>
     </row>
     <row r="6" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>4</v>
-      </c>
-      <c r="B6">
-        <v>6.03</v>
-      </c>
-      <c r="C6">
-        <v>30.59</v>
-      </c>
-      <c r="D6">
-        <v>28.7</v>
-      </c>
-      <c r="E6">
-        <v>20.92</v>
-      </c>
-      <c r="F6">
-        <v>12.29</v>
-      </c>
-      <c r="G6">
-        <v>12.42</v>
-      </c>
-      <c r="H6">
-        <v>4.96</v>
-      </c>
-      <c r="I6">
-        <v>4.07</v>
-      </c>
-      <c r="J6">
-        <v>10.01</v>
-      </c>
-      <c r="K6">
-        <v>11.55</v>
-      </c>
-      <c r="L6">
-        <v>9.31</v>
-      </c>
-      <c r="M6">
-        <v>14.31</v>
-      </c>
-      <c r="N6">
-        <v>143.26</v>
-      </c>
-      <c r="O6">
-        <v>10.53</v>
-      </c>
-      <c r="P6">
-        <v>30.54</v>
-      </c>
-      <c r="Q6">
-        <v>20.92</v>
-      </c>
-      <c r="R6">
-        <v>5.68</v>
+        <v>41</v>
+      </c>
+      <c r="C6" t="s">
+        <v>43</v>
+      </c>
+      <c r="D6" t="s">
+        <v>44</v>
+      </c>
+      <c r="E6" t="s">
+        <v>43</v>
+      </c>
+      <c r="F6" t="s">
+        <v>42</v>
+      </c>
+      <c r="G6" t="s">
+        <v>43</v>
+      </c>
+      <c r="H6" t="s">
+        <v>42</v>
+      </c>
+      <c r="I6" t="s">
+        <v>43</v>
+      </c>
+      <c r="J6" t="s">
+        <v>42</v>
+      </c>
+      <c r="K6" t="s">
+        <v>42</v>
+      </c>
+      <c r="L6" t="s">
+        <v>42</v>
+      </c>
+      <c r="M6" t="s">
+        <v>44</v>
+      </c>
+      <c r="Q6" t="s">
+        <v>43</v>
       </c>
     </row>
     <row r="7" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="B7">
-        <v>61.48</v>
+        <v>0.89</v>
       </c>
       <c r="C7">
-        <v>161.99</v>
+        <v>1.2</v>
       </c>
       <c r="D7">
-        <v>390.26</v>
+        <v>1.34</v>
       </c>
       <c r="E7">
-        <v>3586.11</v>
+        <v>1.94</v>
       </c>
       <c r="F7">
-        <v>2.09</v>
+        <v>0.59</v>
       </c>
       <c r="G7">
-        <v>213.76</v>
+        <v>1.37</v>
       </c>
       <c r="H7">
-        <v>581.12</v>
+        <v>1.5</v>
       </c>
       <c r="I7">
-        <v>4753.76</v>
+        <v>1.28</v>
       </c>
       <c r="J7">
-        <v>81.23</v>
+        <v>1.06</v>
       </c>
       <c r="K7">
-        <v>5021.83</v>
+        <v>1.21</v>
       </c>
       <c r="L7">
-        <v>5021.83</v>
+        <v>0.98</v>
       </c>
       <c r="M7">
-        <v>0.44</v>
+        <v>1.91</v>
       </c>
       <c r="N7">
-        <v>2190.98</v>
+        <v>17.649999999999999</v>
       </c>
       <c r="O7">
-        <v>81.23</v>
+        <v>1.1100000000000001</v>
       </c>
       <c r="P7">
-        <v>390.26</v>
+        <v>1.43</v>
       </c>
       <c r="Q7">
-        <v>3586.11</v>
+        <v>1.94</v>
       </c>
       <c r="R7">
-        <v>4338.8</v>
+        <v>0.78</v>
       </c>
     </row>
     <row r="8" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>29</v>
+        <v>4</v>
       </c>
       <c r="B8">
-        <v>0</v>
+        <v>6.03</v>
       </c>
       <c r="C8">
-        <v>208</v>
+        <v>30.59</v>
       </c>
       <c r="D8">
-        <v>580</v>
+        <v>28.7</v>
       </c>
       <c r="E8">
-        <v>4512</v>
+        <v>20.92</v>
       </c>
       <c r="F8">
-        <v>1774.35</v>
+        <v>12.29</v>
       </c>
       <c r="G8">
-        <v>0</v>
+        <v>12.42</v>
       </c>
       <c r="H8">
-        <v>250.8</v>
+        <v>4.96</v>
       </c>
       <c r="I8">
-        <v>750</v>
+        <v>4.07</v>
       </c>
       <c r="J8">
-        <v>2.65</v>
+        <v>10.01</v>
       </c>
       <c r="K8">
-        <v>2000</v>
+        <v>11.55</v>
       </c>
       <c r="L8">
-        <v>2000</v>
+        <v>9.31</v>
       </c>
       <c r="M8">
-        <v>1090</v>
+        <v>14.31</v>
       </c>
       <c r="N8">
-        <v>0</v>
+        <v>143.26</v>
       </c>
       <c r="O8">
-        <v>2.65</v>
+        <v>10.53</v>
       </c>
       <c r="P8">
-        <v>580</v>
+        <v>30.54</v>
       </c>
       <c r="Q8">
-        <v>4512</v>
+        <v>20.92</v>
       </c>
       <c r="R8">
-        <v>0</v>
+        <v>5.68</v>
       </c>
     </row>
     <row r="9" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
+        <v>5</v>
+      </c>
+      <c r="B9">
+        <v>61.48</v>
+      </c>
+      <c r="C9">
+        <v>161.99</v>
+      </c>
+      <c r="D9">
+        <v>390.26</v>
+      </c>
+      <c r="E9">
+        <v>3586.11</v>
+      </c>
+      <c r="F9">
+        <v>2.09</v>
+      </c>
+      <c r="G9">
+        <v>213.76</v>
+      </c>
+      <c r="H9">
+        <v>581.12</v>
+      </c>
+      <c r="I9">
+        <v>4753.76</v>
+      </c>
+      <c r="J9">
+        <v>81.23</v>
+      </c>
+      <c r="K9">
+        <v>5021.83</v>
+      </c>
+      <c r="L9">
+        <v>5021.83</v>
+      </c>
+      <c r="M9">
+        <v>0.44</v>
+      </c>
+      <c r="N9">
+        <v>2190.98</v>
+      </c>
+      <c r="O9">
+        <v>81.23</v>
+      </c>
+      <c r="P9">
+        <v>390.26</v>
+      </c>
+      <c r="Q9">
+        <v>3586.11</v>
+      </c>
+      <c r="R9">
+        <v>4338.8</v>
+      </c>
+    </row>
+    <row r="10" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>29</v>
+      </c>
+      <c r="B10">
+        <v>0</v>
+      </c>
+      <c r="C10">
+        <v>208</v>
+      </c>
+      <c r="D10">
+        <v>580</v>
+      </c>
+      <c r="E10">
+        <v>4512</v>
+      </c>
+      <c r="F10">
+        <v>1774.35</v>
+      </c>
+      <c r="G10">
+        <v>0</v>
+      </c>
+      <c r="H10">
+        <v>250.8</v>
+      </c>
+      <c r="I10">
+        <v>750</v>
+      </c>
+      <c r="J10">
+        <v>2.65</v>
+      </c>
+      <c r="K10">
+        <v>2000</v>
+      </c>
+      <c r="L10">
+        <v>2000</v>
+      </c>
+      <c r="M10">
+        <v>1090</v>
+      </c>
+      <c r="N10">
+        <v>0</v>
+      </c>
+      <c r="O10">
+        <v>2.65</v>
+      </c>
+      <c r="P10">
+        <v>580</v>
+      </c>
+      <c r="Q10">
+        <v>4512</v>
+      </c>
+      <c r="R10">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
         <v>24</v>
       </c>
-      <c r="B9" s="2" t="s">
+      <c r="B11" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="C9" s="2" t="s">
+      <c r="C11" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="D9" s="2" t="s">
+      <c r="D11" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="E9" s="2" t="s">
+      <c r="E11" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="F9" s="2" t="s">
+      <c r="F11" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="G9" s="2" t="s">
+      <c r="G11" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="H9" s="2" t="s">
+      <c r="H11" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="I9" s="2" t="s">
+      <c r="I11" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="J9" s="2" t="s">
+      <c r="J11" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="K9" s="2" t="s">
+      <c r="K11" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="L9" s="2" t="s">
+      <c r="L11" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="M9" s="2" t="s">
+      <c r="M11" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="N9" s="2" t="s">
+      <c r="N11" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="O9" s="2" t="s">
+      <c r="O11" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="P9" s="2" t="s">
+      <c r="P11" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="Q9" s="2" t="s">
+      <c r="Q11" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="R9" s="2" t="s">
+      <c r="R11" s="2" t="s">
         <v>39</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="D9" r:id="rId1" xr:uid="{548C98B5-F3E3-4700-BC84-FF4F5138811A}"/>
-    <hyperlink ref="C9" r:id="rId2" xr:uid="{2DA283A4-C6EA-40D6-939F-D22B30E7B883}"/>
-    <hyperlink ref="B9" r:id="rId3" location="resumen" xr:uid="{C166E8DB-3625-4D6A-9964-64727C287454}"/>
-    <hyperlink ref="E9" r:id="rId4" xr:uid="{D521BBBB-DA1E-4CB1-912A-F4C5AD9F4F7C}"/>
-    <hyperlink ref="F9" r:id="rId5" xr:uid="{DA028F1D-F28B-460C-A841-E9D2EC39570E}"/>
-    <hyperlink ref="I9" r:id="rId6" xr:uid="{54B27BCE-633F-44E3-BD26-F4588777EADD}"/>
-    <hyperlink ref="J9" r:id="rId7" location="resumen" xr:uid="{A76F462E-61B5-432B-9FEA-AAD7496B1091}"/>
-    <hyperlink ref="K9" r:id="rId8" xr:uid="{3E235CBF-9071-4F8C-BEBF-36FE0401D3E1}"/>
-    <hyperlink ref="L9" r:id="rId9" xr:uid="{6C73B067-55C0-4BAD-AA1D-08559EFC33B2}"/>
-    <hyperlink ref="M9" r:id="rId10" location="resumen" xr:uid="{1037CDC5-35DC-4373-950D-1A5B71DC7824}"/>
-    <hyperlink ref="N9" r:id="rId11" xr:uid="{838B76B2-5760-4137-8E4B-CD1D36F21391}"/>
-    <hyperlink ref="H9" r:id="rId12" xr:uid="{21A7C0D0-E3F2-4A5A-9CC1-19F202657C3D}"/>
-    <hyperlink ref="G9" r:id="rId13" xr:uid="{7E225246-03C7-43DB-82FA-8EA312EEA4F1}"/>
-    <hyperlink ref="O9" r:id="rId14" xr:uid="{DF390B55-2E70-42A6-ADBF-9C0B4FBE5502}"/>
-    <hyperlink ref="P9" r:id="rId15" xr:uid="{895F1DEC-3582-4116-A9C2-10321F6E3214}"/>
-    <hyperlink ref="Q9" r:id="rId16" xr:uid="{29ACF7C6-5021-4673-8052-7C3731191E29}"/>
-    <hyperlink ref="R9" r:id="rId17" xr:uid="{58A99770-EA64-4E41-98DC-82BA23B70E4A}"/>
+    <hyperlink ref="D11" r:id="rId1" xr:uid="{548C98B5-F3E3-4700-BC84-FF4F5138811A}"/>
+    <hyperlink ref="C11" r:id="rId2" xr:uid="{2DA283A4-C6EA-40D6-939F-D22B30E7B883}"/>
+    <hyperlink ref="B11" r:id="rId3" location="resumen" xr:uid="{C166E8DB-3625-4D6A-9964-64727C287454}"/>
+    <hyperlink ref="E11" r:id="rId4" xr:uid="{D521BBBB-DA1E-4CB1-912A-F4C5AD9F4F7C}"/>
+    <hyperlink ref="F11" r:id="rId5" xr:uid="{DA028F1D-F28B-460C-A841-E9D2EC39570E}"/>
+    <hyperlink ref="I11" r:id="rId6" xr:uid="{54B27BCE-633F-44E3-BD26-F4588777EADD}"/>
+    <hyperlink ref="J11" r:id="rId7" location="resumen" xr:uid="{A76F462E-61B5-432B-9FEA-AAD7496B1091}"/>
+    <hyperlink ref="K11" r:id="rId8" xr:uid="{3E235CBF-9071-4F8C-BEBF-36FE0401D3E1}"/>
+    <hyperlink ref="L11" r:id="rId9" xr:uid="{6C73B067-55C0-4BAD-AA1D-08559EFC33B2}"/>
+    <hyperlink ref="M11" r:id="rId10" location="resumen" xr:uid="{1037CDC5-35DC-4373-950D-1A5B71DC7824}"/>
+    <hyperlink ref="N11" r:id="rId11" xr:uid="{838B76B2-5760-4137-8E4B-CD1D36F21391}"/>
+    <hyperlink ref="H11" r:id="rId12" xr:uid="{21A7C0D0-E3F2-4A5A-9CC1-19F202657C3D}"/>
+    <hyperlink ref="G11" r:id="rId13" xr:uid="{7E225246-03C7-43DB-82FA-8EA312EEA4F1}"/>
+    <hyperlink ref="O11" r:id="rId14" xr:uid="{DF390B55-2E70-42A6-ADBF-9C0B4FBE5502}"/>
+    <hyperlink ref="P11" r:id="rId15" xr:uid="{895F1DEC-3582-4116-A9C2-10321F6E3214}"/>
+    <hyperlink ref="Q11" r:id="rId16" xr:uid="{29ACF7C6-5021-4673-8052-7C3731191E29}"/>
+    <hyperlink ref="R11" r:id="rId17" xr:uid="{58A99770-EA64-4E41-98DC-82BA23B70E4A}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>